<commit_message>
update BM KPH CTD
</commit_message>
<xml_diff>
--- a/dataproduct.api/wwwroot/templates/BM_TongHopPhieuSanPhamKPH.xlsx
+++ b/dataproduct.api/wwwroot/templates/BM_TongHopPhieuSanPhamKPH.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Software\03. ThongKePKH\DATAPRODUCT_V2\dataproduct.api\dataproduct.api\wwwroot\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FDF1B32-85D3-4666-9EB0-EE9F40D418B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{669B03A5-380C-4620-BFC0-15C8C4C99D84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{77908C05-ABC3-4C3F-A6F5-1B05425144FB}"/>
   </bookViews>
@@ -357,6 +357,39 @@
     <xf numFmtId="0" fontId="9" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -398,39 +431,6 @@
     </xf>
     <xf numFmtId="164" fontId="6" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -790,7 +790,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{43BAB014-E6DF-4BFD-BF20-A00AB0E3B9F2}">
-  <dimension ref="A1:AB31"/>
+  <dimension ref="A1:AB9"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.5703125" style="1" customWidth="1"/>
@@ -821,186 +821,186 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="28"/>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
+      <c r="A1" s="14"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
       <c r="E1" s="11"/>
     </row>
     <row r="2" spans="1:28" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="28"/>
-      <c r="B2" s="28"/>
-      <c r="C2" s="28"/>
-      <c r="D2" s="28"/>
+      <c r="A2" s="14"/>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
       <c r="E2" s="11"/>
     </row>
     <row r="3" spans="1:28" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A3" s="29" t="s">
+      <c r="A3" s="22" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="29"/>
-      <c r="C3" s="29"/>
-      <c r="D3" s="29"/>
-      <c r="E3" s="29"/>
-      <c r="F3" s="29"/>
-      <c r="G3" s="29"/>
-      <c r="H3" s="29"/>
-      <c r="I3" s="29"/>
-      <c r="J3" s="29"/>
-      <c r="K3" s="29"/>
-      <c r="L3" s="29"/>
-      <c r="M3" s="29"/>
-      <c r="N3" s="29"/>
-      <c r="O3" s="29"/>
-      <c r="P3" s="29"/>
-      <c r="Q3" s="29"/>
-      <c r="R3" s="29"/>
-      <c r="S3" s="29"/>
-      <c r="T3" s="29"/>
-      <c r="U3" s="29"/>
-      <c r="V3" s="29"/>
-      <c r="W3" s="29"/>
-      <c r="X3" s="29"/>
-      <c r="Y3" s="29"/>
-      <c r="Z3" s="29"/>
-      <c r="AA3" s="29"/>
-      <c r="AB3" s="29"/>
+      <c r="B3" s="22"/>
+      <c r="C3" s="22"/>
+      <c r="D3" s="22"/>
+      <c r="E3" s="22"/>
+      <c r="F3" s="22"/>
+      <c r="G3" s="22"/>
+      <c r="H3" s="22"/>
+      <c r="I3" s="22"/>
+      <c r="J3" s="22"/>
+      <c r="K3" s="22"/>
+      <c r="L3" s="22"/>
+      <c r="M3" s="22"/>
+      <c r="N3" s="22"/>
+      <c r="O3" s="22"/>
+      <c r="P3" s="22"/>
+      <c r="Q3" s="22"/>
+      <c r="R3" s="22"/>
+      <c r="S3" s="22"/>
+      <c r="T3" s="22"/>
+      <c r="U3" s="22"/>
+      <c r="V3" s="22"/>
+      <c r="W3" s="22"/>
+      <c r="X3" s="22"/>
+      <c r="Y3" s="22"/>
+      <c r="Z3" s="22"/>
+      <c r="AA3" s="22"/>
+      <c r="AB3" s="22"/>
     </row>
     <row r="4" spans="1:28" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="30" t="s">
+      <c r="A4" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="30"/>
-      <c r="C4" s="30"/>
-      <c r="D4" s="30"/>
-      <c r="E4" s="30"/>
-      <c r="F4" s="30"/>
-      <c r="G4" s="30"/>
-      <c r="H4" s="30"/>
-      <c r="I4" s="30"/>
-      <c r="J4" s="30"/>
-      <c r="K4" s="30"/>
-      <c r="L4" s="30"/>
-      <c r="M4" s="30"/>
-      <c r="N4" s="30"/>
-      <c r="O4" s="30"/>
-      <c r="P4" s="30"/>
-      <c r="Q4" s="30"/>
-      <c r="R4" s="30"/>
-      <c r="S4" s="30"/>
-      <c r="T4" s="30"/>
-      <c r="U4" s="30"/>
-      <c r="V4" s="30"/>
-      <c r="W4" s="30"/>
-      <c r="X4" s="30"/>
-      <c r="Y4" s="30"/>
-      <c r="Z4" s="30"/>
-      <c r="AA4" s="30"/>
-      <c r="AB4" s="30"/>
+      <c r="B4" s="23"/>
+      <c r="C4" s="23"/>
+      <c r="D4" s="23"/>
+      <c r="E4" s="23"/>
+      <c r="F4" s="23"/>
+      <c r="G4" s="23"/>
+      <c r="H4" s="23"/>
+      <c r="I4" s="23"/>
+      <c r="J4" s="23"/>
+      <c r="K4" s="23"/>
+      <c r="L4" s="23"/>
+      <c r="M4" s="23"/>
+      <c r="N4" s="23"/>
+      <c r="O4" s="23"/>
+      <c r="P4" s="23"/>
+      <c r="Q4" s="23"/>
+      <c r="R4" s="23"/>
+      <c r="S4" s="23"/>
+      <c r="T4" s="23"/>
+      <c r="U4" s="23"/>
+      <c r="V4" s="23"/>
+      <c r="W4" s="23"/>
+      <c r="X4" s="23"/>
+      <c r="Y4" s="23"/>
+      <c r="Z4" s="23"/>
+      <c r="AA4" s="23"/>
+      <c r="AB4" s="23"/>
     </row>
     <row r="5" spans="1:28" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3"/>
     </row>
     <row r="6" spans="1:28" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="27" t="s">
+      <c r="A6" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B6" s="27" t="s">
+      <c r="B6" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="32" t="s">
+      <c r="C6" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="D6" s="32" t="s">
+      <c r="D6" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="E6" s="35" t="s">
+      <c r="E6" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="F6" s="27" t="s">
+      <c r="F6" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="G6" s="27" t="s">
+      <c r="G6" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="H6" s="34" t="s">
+      <c r="H6" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="I6" s="13" t="s">
+      <c r="I6" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="J6" s="19" t="s">
+      <c r="J6" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="K6" s="20"/>
-      <c r="L6" s="20"/>
-      <c r="M6" s="20"/>
-      <c r="N6" s="20"/>
-      <c r="O6" s="20"/>
-      <c r="P6" s="20"/>
-      <c r="Q6" s="20"/>
-      <c r="R6" s="23" t="s">
+      <c r="K6" s="31"/>
+      <c r="L6" s="31"/>
+      <c r="M6" s="31"/>
+      <c r="N6" s="31"/>
+      <c r="O6" s="31"/>
+      <c r="P6" s="31"/>
+      <c r="Q6" s="31"/>
+      <c r="R6" s="34" t="s">
         <v>21</v>
       </c>
-      <c r="S6" s="24" t="s">
+      <c r="S6" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="T6" s="19" t="s">
+      <c r="T6" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="U6" s="20"/>
-      <c r="V6" s="20"/>
-      <c r="W6" s="20"/>
-      <c r="X6" s="20"/>
-      <c r="Y6" s="20"/>
-      <c r="Z6" s="20"/>
-      <c r="AA6" s="16" t="s">
+      <c r="U6" s="31"/>
+      <c r="V6" s="31"/>
+      <c r="W6" s="31"/>
+      <c r="X6" s="31"/>
+      <c r="Y6" s="31"/>
+      <c r="Z6" s="31"/>
+      <c r="AA6" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="AB6" s="13" t="s">
+      <c r="AB6" s="24" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:28" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="31"/>
-      <c r="B7" s="31"/>
-      <c r="C7" s="33"/>
-      <c r="D7" s="33"/>
-      <c r="E7" s="36"/>
-      <c r="F7" s="31"/>
-      <c r="G7" s="27"/>
-      <c r="H7" s="34"/>
-      <c r="I7" s="14"/>
-      <c r="J7" s="21"/>
-      <c r="K7" s="22"/>
-      <c r="L7" s="22"/>
-      <c r="M7" s="22"/>
-      <c r="N7" s="22"/>
-      <c r="O7" s="22"/>
-      <c r="P7" s="22"/>
-      <c r="Q7" s="22"/>
-      <c r="R7" s="23"/>
-      <c r="S7" s="25"/>
-      <c r="T7" s="21"/>
-      <c r="U7" s="22"/>
-      <c r="V7" s="22"/>
-      <c r="W7" s="22"/>
-      <c r="X7" s="22"/>
-      <c r="Y7" s="22"/>
-      <c r="Z7" s="22"/>
-      <c r="AA7" s="17"/>
-      <c r="AB7" s="14"/>
+      <c r="A7" s="15"/>
+      <c r="B7" s="15"/>
+      <c r="C7" s="17"/>
+      <c r="D7" s="17"/>
+      <c r="E7" s="20"/>
+      <c r="F7" s="15"/>
+      <c r="G7" s="13"/>
+      <c r="H7" s="18"/>
+      <c r="I7" s="25"/>
+      <c r="J7" s="32"/>
+      <c r="K7" s="33"/>
+      <c r="L7" s="33"/>
+      <c r="M7" s="33"/>
+      <c r="N7" s="33"/>
+      <c r="O7" s="33"/>
+      <c r="P7" s="33"/>
+      <c r="Q7" s="33"/>
+      <c r="R7" s="34"/>
+      <c r="S7" s="36"/>
+      <c r="T7" s="32"/>
+      <c r="U7" s="33"/>
+      <c r="V7" s="33"/>
+      <c r="W7" s="33"/>
+      <c r="X7" s="33"/>
+      <c r="Y7" s="33"/>
+      <c r="Z7" s="33"/>
+      <c r="AA7" s="28"/>
+      <c r="AB7" s="25"/>
     </row>
     <row r="8" spans="1:28" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="31"/>
-      <c r="B8" s="31"/>
-      <c r="C8" s="33"/>
-      <c r="D8" s="33"/>
-      <c r="E8" s="37"/>
-      <c r="F8" s="31"/>
-      <c r="G8" s="27"/>
-      <c r="H8" s="34"/>
-      <c r="I8" s="15"/>
+      <c r="A8" s="15"/>
+      <c r="B8" s="15"/>
+      <c r="C8" s="17"/>
+      <c r="D8" s="17"/>
+      <c r="E8" s="21"/>
+      <c r="F8" s="15"/>
+      <c r="G8" s="13"/>
+      <c r="H8" s="18"/>
+      <c r="I8" s="26"/>
       <c r="J8" s="4" t="s">
         <v>15</v>
       </c>
@@ -1025,8 +1025,8 @@
       <c r="Q8" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="R8" s="23"/>
-      <c r="S8" s="26"/>
+      <c r="R8" s="34"/>
+      <c r="S8" s="37"/>
       <c r="T8" s="4" t="s">
         <v>15</v>
       </c>
@@ -1048,10 +1048,10 @@
       <c r="Z8" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="AA8" s="18"/>
-      <c r="AB8" s="15"/>
+      <c r="AA8" s="29"/>
+      <c r="AB8" s="26"/>
     </row>
-    <row r="9" spans="1:28" ht="69" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:28" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A9" s="5"/>
       <c r="B9" s="6"/>
       <c r="C9" s="7"/>
@@ -1081,37 +1081,8 @@
       <c r="AA9" s="8"/>
       <c r="AB9" s="9"/>
     </row>
-    <row r="10" spans="1:28" ht="44.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="11" spans="1:28" ht="44.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="12" spans="1:28" ht="44.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="13" spans="1:28" ht="44.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="14" spans="1:28" ht="44.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="15" spans="1:28" ht="44.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="16" spans="1:28" ht="44.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="17" ht="44.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="18" ht="44.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="19" ht="44.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="20" ht="44.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="21" ht="44.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="22" ht="44.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="23" ht="44.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="24" ht="44.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="25" ht="44.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="26" ht="44.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="27" ht="44.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="28" ht="44.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="29" ht="44.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="30" ht="44.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="31" ht="44.25" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="G6:G8"/>
-    <mergeCell ref="A1:D2"/>
-    <mergeCell ref="A6:A8"/>
-    <mergeCell ref="B6:B8"/>
-    <mergeCell ref="C6:C8"/>
-    <mergeCell ref="D6:D8"/>
-    <mergeCell ref="F6:F8"/>
     <mergeCell ref="H6:H8"/>
     <mergeCell ref="E6:E8"/>
     <mergeCell ref="A3:AB3"/>
@@ -1123,6 +1094,13 @@
     <mergeCell ref="R6:R8"/>
     <mergeCell ref="S6:S8"/>
     <mergeCell ref="T6:Z7"/>
+    <mergeCell ref="G6:G8"/>
+    <mergeCell ref="A1:D2"/>
+    <mergeCell ref="A6:A8"/>
+    <mergeCell ref="B6:B8"/>
+    <mergeCell ref="C6:C8"/>
+    <mergeCell ref="D6:D8"/>
+    <mergeCell ref="F6:F8"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1306,20 +1284,20 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="7bdf782f-2886-4011-99ee-a2495b2dfaf9" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="7bdf782f-2886-4011-99ee-a2495b2dfaf9" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1341,6 +1319,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{24B1C2B3-91A9-494D-BEB6-2B1BB33BE342}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{847D81C1-0646-4BD0-BC63-D9DF50568213}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="7bdf782f-2886-4011-99ee-a2495b2dfaf9"/>
@@ -1354,12 +1340,4 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{24B1C2B3-91A9-494D-BEB6-2B1BB33BE342}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>